<commit_message>
Malu & Girija Ammayi sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Sep26.xlsx
+++ b/docs/Chiraath-Summary-Sep26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCD8975-8CC4-F64C-B123-64873FC64FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6F738AE-F557-3C4C-BF9C-52A1425C6E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3446" uniqueCount="1368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3457" uniqueCount="1371">
   <si>
     <t>Notes:</t>
   </si>
@@ -3895,9 +3895,6 @@
     <t>DTDC parcel charges</t>
   </si>
   <si>
-    <t>Ranju Bank Staff (850)</t>
-  </si>
-  <si>
     <t>Gracy Kunjumon</t>
   </si>
   <si>
@@ -4139,9 +4136,6 @@
     <t>Thresiamma</t>
   </si>
   <si>
-    <t>CHR-207 - Violet/Mustard</t>
-  </si>
-  <si>
     <t>Navy/blue, yellow/peacock blue, turquoise/violet</t>
   </si>
   <si>
@@ -4167,6 +4161,21 @@
   </si>
   <si>
     <t>Latha Ammayi - Maroon, Blue returned</t>
+  </si>
+  <si>
+    <t>Malu, Girija</t>
+  </si>
+  <si>
+    <t>CHR-243 - leaf design blue</t>
+  </si>
+  <si>
+    <t>CHR-207 - Violet/Mustard, CHR-193 - navy</t>
+  </si>
+  <si>
+    <t>Girija Ammayi</t>
+  </si>
+  <si>
+    <t>CHR-243 - leaf design Red</t>
   </si>
 </sst>
 </file>
@@ -5074,7 +5083,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>360</c:v>
+                  <c:v>361</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>99</c:v>
@@ -5177,7 +5186,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>180</c:v>
+                  <c:v>179</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>65</c:v>
@@ -5510,7 +5519,7 @@
                   <c:v>69573</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>128214.14666666667</c:v>
+                  <c:v>127669.14666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -6006,7 +6015,7 @@
                   <c:v>65156</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>78068</c:v>
+                  <c:v>79568</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6446,7 +6455,7 @@
                   <c:v>-37044</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>32220</c:v>
+                  <c:v>33720</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6907,10 +6916,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>464</c:v>
+                  <c:v>465</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>266</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8117,7 +8126,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>548551</v>
+        <v>552551</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -8134,7 +8143,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>571491</v>
+        <v>572991</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -8151,7 +8160,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-53644</v>
+        <v>-49644</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -8363,15 +8372,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>479698</v>
+        <v>483698</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>182886.90339999998</v>
+        <v>184220.50339999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>296811.09660000005</v>
+        <v>299477.49660000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8379,11 +8388,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>159501.07060000004</v>
+        <v>162167.4706</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹159,501</v>
+        <v>Pay ₹162,167</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8397,11 +8406,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>182777.19320000001</v>
+        <v>184109.9932</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-127454.19320000001</v>
+        <v>-128786.9932</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8409,11 +8418,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-55867.151200000008</v>
+        <v>-57199.951199999996</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹55,867</v>
+        <v>Receive ₹57,200</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8427,11 +8436,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>182886.90339999998</v>
+        <v>184220.50339999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-170356.90339999998</v>
+        <v>-171690.50339999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8439,11 +8448,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-104633.91939999997</v>
+        <v>-105967.51939999998</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹104,634</v>
+        <v>Receive ₹105,968</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8571,7 +8580,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>548551</v>
+        <v>552551</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8580,14 +8589,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-53644</v>
+        <v>-49644</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>189190.34666666665</v>
+        <v>188645.34666666665</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8639,7 +8648,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>464</v>
+        <v>465</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8663,7 +8672,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8761,11 +8770,11 @@
       </c>
       <c r="C17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A17)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>78068</v>
+        <v>79568</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>32220</v>
+        <v>33720</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1">
@@ -8859,11 +8868,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8890,7 +8899,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$476=J48)*(INVENTORY!$D$2:$D$476)*(INVENTORY!$G$2:$G$476))</f>
-        <v>128214.14666666667</v>
+        <v>127669.14666666667</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -10529,7 +10538,7 @@
         <v>3046</v>
       </c>
       <c r="D110" s="36" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="111" spans="1:4" ht="15" customHeight="1">
@@ -12605,7 +12614,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:I328"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
@@ -12650,7 +12658,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14" hidden="1">
+    <row r="2" spans="1:9" ht="14">
       <c r="A2" s="82">
         <v>45900</v>
       </c>
@@ -12673,7 +12681,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="14" hidden="1">
+    <row r="3" spans="1:9" ht="14">
       <c r="A3" s="84">
         <v>45900</v>
       </c>
@@ -12696,7 +12704,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="14" hidden="1">
+    <row r="4" spans="1:9" ht="14">
       <c r="A4" s="82">
         <v>45900</v>
       </c>
@@ -12719,7 +12727,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14" hidden="1">
+    <row r="5" spans="1:9" ht="14">
       <c r="A5" s="84">
         <v>45900</v>
       </c>
@@ -12765,7 +12773,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="14" hidden="1">
+    <row r="7" spans="1:9" ht="14">
       <c r="A7" s="84">
         <v>45900</v>
       </c>
@@ -12788,7 +12796,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14" hidden="1">
+    <row r="8" spans="1:9" ht="14">
       <c r="A8" s="82">
         <v>45900</v>
       </c>
@@ -12811,7 +12819,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="14" hidden="1">
+    <row r="9" spans="1:9" ht="14">
       <c r="A9" s="84">
         <v>45901</v>
       </c>
@@ -12834,7 +12842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="14" hidden="1">
+    <row r="10" spans="1:9" ht="14">
       <c r="A10" s="82">
         <v>45902</v>
       </c>
@@ -12857,7 +12865,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14" hidden="1">
+    <row r="11" spans="1:9" ht="14">
       <c r="A11" s="84">
         <v>45903</v>
       </c>
@@ -12880,7 +12888,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="14" hidden="1">
+    <row r="12" spans="1:9" ht="14">
       <c r="A12" s="82">
         <v>45904</v>
       </c>
@@ -12903,7 +12911,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="14" hidden="1">
+    <row r="13" spans="1:9" ht="14">
       <c r="A13" s="84">
         <v>45905</v>
       </c>
@@ -12926,7 +12934,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14" hidden="1">
+    <row r="14" spans="1:9" ht="14">
       <c r="A14" s="82">
         <v>45906</v>
       </c>
@@ -12949,7 +12957,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="14" hidden="1">
+    <row r="15" spans="1:9" ht="14">
       <c r="A15" s="84">
         <v>45907</v>
       </c>
@@ -12972,7 +12980,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="14" hidden="1">
+    <row r="16" spans="1:9" ht="14">
       <c r="A16" s="82">
         <v>45908</v>
       </c>
@@ -12995,7 +13003,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="14" hidden="1">
+    <row r="17" spans="1:9" ht="14">
       <c r="A17" s="84">
         <v>45909</v>
       </c>
@@ -13018,7 +13026,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14" hidden="1">
+    <row r="18" spans="1:9" ht="14">
       <c r="A18" s="82">
         <v>45910</v>
       </c>
@@ -13041,7 +13049,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="14" hidden="1">
+    <row r="19" spans="1:9" ht="14">
       <c r="A19" s="84">
         <v>45911</v>
       </c>
@@ -13064,7 +13072,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="14" hidden="1">
+    <row r="20" spans="1:9" ht="14">
       <c r="A20" s="82">
         <v>45912</v>
       </c>
@@ -13087,7 +13095,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="14" hidden="1">
+    <row r="21" spans="1:9" ht="14">
       <c r="A21" s="84">
         <v>45913</v>
       </c>
@@ -13110,7 +13118,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="14" hidden="1">
+    <row r="22" spans="1:9" ht="14">
       <c r="A22" s="82">
         <v>45914</v>
       </c>
@@ -13133,7 +13141,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="14" hidden="1">
+    <row r="23" spans="1:9" ht="14">
       <c r="A23" s="84">
         <v>45915</v>
       </c>
@@ -13156,7 +13164,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14" hidden="1">
+    <row r="24" spans="1:9" ht="14">
       <c r="A24" s="82">
         <v>45916</v>
       </c>
@@ -13179,7 +13187,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="14" hidden="1">
+    <row r="25" spans="1:9" ht="14">
       <c r="A25" s="84">
         <v>45917</v>
       </c>
@@ -13202,7 +13210,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="14" hidden="1">
+    <row r="26" spans="1:9" ht="14">
       <c r="A26" s="82">
         <v>45917</v>
       </c>
@@ -13225,7 +13233,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="14" hidden="1">
+    <row r="27" spans="1:9" ht="14">
       <c r="A27" s="84">
         <v>45918</v>
       </c>
@@ -13248,7 +13256,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="14" hidden="1">
+    <row r="28" spans="1:9" ht="14">
       <c r="A28" s="82">
         <v>45919</v>
       </c>
@@ -13271,7 +13279,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="14" hidden="1">
+    <row r="29" spans="1:9" ht="14">
       <c r="A29" s="84">
         <v>45920</v>
       </c>
@@ -13294,7 +13302,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="14" hidden="1">
+    <row r="30" spans="1:9" ht="14">
       <c r="A30" s="82">
         <v>45921</v>
       </c>
@@ -13317,7 +13325,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="14" hidden="1">
+    <row r="31" spans="1:9" ht="14">
       <c r="A31" s="84">
         <v>45922</v>
       </c>
@@ -13340,7 +13348,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="14" hidden="1">
+    <row r="32" spans="1:9" ht="14">
       <c r="A32" s="82">
         <v>45924</v>
       </c>
@@ -13363,7 +13371,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="14" hidden="1">
+    <row r="33" spans="1:9" ht="14">
       <c r="A33" s="84">
         <v>45924</v>
       </c>
@@ -13386,7 +13394,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="14" hidden="1">
+    <row r="34" spans="1:9" ht="14">
       <c r="A34" s="82">
         <v>45930</v>
       </c>
@@ -13409,7 +13417,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="14" hidden="1">
+    <row r="35" spans="1:9" ht="14">
       <c r="A35" s="84">
         <v>45933.931944444397</v>
       </c>
@@ -13432,7 +13440,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="14" hidden="1">
+    <row r="36" spans="1:9" ht="14">
       <c r="A36" s="82">
         <v>45934.931944386597</v>
       </c>
@@ -13455,7 +13463,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="14" hidden="1">
+    <row r="37" spans="1:9" ht="14">
       <c r="A37" s="84">
         <v>45935.931944386597</v>
       </c>
@@ -13478,7 +13486,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="14" hidden="1">
+    <row r="38" spans="1:9" ht="14">
       <c r="A38" s="82">
         <v>45939.931944444397</v>
       </c>
@@ -13501,7 +13509,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="14" hidden="1">
+    <row r="39" spans="1:9" ht="14">
       <c r="A39" s="84">
         <v>45939.931944444397</v>
       </c>
@@ -13524,7 +13532,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="14" hidden="1">
+    <row r="40" spans="1:9" ht="14">
       <c r="A40" s="82">
         <v>45945</v>
       </c>
@@ -13547,7 +13555,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="14" hidden="1">
+    <row r="41" spans="1:9" ht="14">
       <c r="A41" s="84">
         <v>45946</v>
       </c>
@@ -13570,7 +13578,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="14" hidden="1">
+    <row r="42" spans="1:9" ht="14">
       <c r="A42" s="82">
         <v>45946</v>
       </c>
@@ -13593,7 +13601,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="14" hidden="1">
+    <row r="43" spans="1:9" ht="14">
       <c r="A43" s="84">
         <v>45947</v>
       </c>
@@ -13616,7 +13624,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="14" hidden="1">
+    <row r="44" spans="1:9" ht="14">
       <c r="A44" s="82">
         <v>45948</v>
       </c>
@@ -13639,7 +13647,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="14" hidden="1">
+    <row r="45" spans="1:9" ht="14">
       <c r="A45" s="84">
         <v>45949</v>
       </c>
@@ -13662,7 +13670,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="14" hidden="1">
+    <row r="46" spans="1:9" ht="14">
       <c r="A46" s="82">
         <v>45950</v>
       </c>
@@ -13685,7 +13693,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="14" hidden="1">
+    <row r="47" spans="1:9" ht="14">
       <c r="A47" s="84">
         <v>45951</v>
       </c>
@@ -13708,7 +13716,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="14" hidden="1">
+    <row r="48" spans="1:9" ht="14">
       <c r="A48" s="82">
         <v>45964</v>
       </c>
@@ -13731,7 +13739,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="14" hidden="1">
+    <row r="49" spans="1:9" ht="14">
       <c r="A49" s="84">
         <v>45963</v>
       </c>
@@ -13754,7 +13762,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="14" hidden="1">
+    <row r="50" spans="1:9" ht="14">
       <c r="A50" s="82">
         <v>45982</v>
       </c>
@@ -13777,7 +13785,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="14" hidden="1">
+    <row r="51" spans="1:9" ht="14">
       <c r="A51" s="84">
         <v>45983</v>
       </c>
@@ -13800,7 +13808,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="14" hidden="1">
+    <row r="52" spans="1:9" ht="14">
       <c r="A52" s="82">
         <v>45984</v>
       </c>
@@ -13823,7 +13831,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="14" hidden="1">
+    <row r="53" spans="1:9" ht="14">
       <c r="A53" s="84">
         <v>45985</v>
       </c>
@@ -13846,7 +13854,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="54" spans="1:9" ht="13.5" customHeight="1">
       <c r="A54" s="82">
         <v>45986</v>
       </c>
@@ -13871,7 +13879,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="55" spans="1:9" ht="15.75" customHeight="1">
       <c r="A55" s="84">
         <v>45992</v>
       </c>
@@ -13896,7 +13904,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="56" spans="1:9" ht="13.5" customHeight="1">
       <c r="A56" s="82">
         <v>45992</v>
       </c>
@@ -13921,7 +13929,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="57" spans="1:9" ht="15.75" customHeight="1">
       <c r="A57" s="84">
         <v>45996</v>
       </c>
@@ -13946,7 +13954,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="58" spans="1:9" ht="42" customHeight="1">
       <c r="A58" s="82">
         <v>45996</v>
       </c>
@@ -13971,7 +13979,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="59" spans="1:9" ht="15.75" customHeight="1">
       <c r="A59" s="84">
         <v>45996</v>
       </c>
@@ -13996,7 +14004,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="60" spans="1:9" ht="13.5" customHeight="1">
       <c r="A60" s="82">
         <v>46007</v>
       </c>
@@ -14021,7 +14029,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="61" spans="1:9" ht="15.75" customHeight="1">
       <c r="A61" s="84">
         <v>46008</v>
       </c>
@@ -14048,7 +14056,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="62" spans="1:9" ht="13.5" customHeight="1">
       <c r="A62" s="82">
         <v>46008</v>
       </c>
@@ -14073,7 +14081,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="63" spans="1:9" ht="15.75" customHeight="1">
       <c r="A63" s="84">
         <v>46008</v>
       </c>
@@ -14098,7 +14106,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="64" spans="1:9" ht="15.75" customHeight="1">
       <c r="A64" s="84">
         <v>46008</v>
       </c>
@@ -14123,7 +14131,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="65" spans="1:9" ht="13.5" customHeight="1">
       <c r="A65" s="82">
         <v>46009</v>
       </c>
@@ -14148,7 +14156,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="66" spans="1:9" ht="15.75" customHeight="1">
       <c r="A66" s="84">
         <v>46010</v>
       </c>
@@ -14173,7 +14181,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="67" spans="1:9" ht="13.5" customHeight="1">
       <c r="A67" s="82">
         <v>46010</v>
       </c>
@@ -14200,7 +14208,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="31.5" hidden="1" customHeight="1">
+    <row r="68" spans="1:9" ht="31.5" customHeight="1">
       <c r="A68" s="84">
         <v>46011</v>
       </c>
@@ -14225,7 +14233,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="69" spans="1:9" ht="13.5" customHeight="1">
       <c r="A69" s="82">
         <v>46011</v>
       </c>
@@ -14250,7 +14258,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="70" spans="1:9" ht="13.5" customHeight="1">
       <c r="A70" s="82">
         <v>46011</v>
       </c>
@@ -14275,7 +14283,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="71" spans="1:9" ht="15.75" customHeight="1">
       <c r="A71" s="84">
         <v>46011</v>
       </c>
@@ -14300,7 +14308,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="72" spans="1:9" ht="27.75" customHeight="1">
       <c r="A72" s="82">
         <v>46011</v>
       </c>
@@ -14325,7 +14333,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="31.5" hidden="1" customHeight="1">
+    <row r="73" spans="1:9" ht="31.5" customHeight="1">
       <c r="A73" s="84">
         <v>46011</v>
       </c>
@@ -14350,7 +14358,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="74" spans="1:9" ht="13.5" customHeight="1">
       <c r="A74" s="82">
         <v>46013</v>
       </c>
@@ -14377,7 +14385,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="75" spans="1:9" ht="15.75" customHeight="1">
       <c r="A75" s="84">
         <v>46013</v>
       </c>
@@ -14402,7 +14410,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="76" spans="1:9" ht="15.75" customHeight="1">
       <c r="A76" s="84">
         <v>46017</v>
       </c>
@@ -14427,7 +14435,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="77" spans="1:9" ht="13.5" customHeight="1">
       <c r="A77" s="82">
         <v>46017</v>
       </c>
@@ -14452,7 +14460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="78" spans="1:9" ht="15.75" customHeight="1">
       <c r="A78" s="84">
         <v>46017</v>
       </c>
@@ -14477,7 +14485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="79" spans="1:9" ht="13.5" customHeight="1">
       <c r="A79" s="82">
         <v>46017</v>
       </c>
@@ -14502,7 +14510,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="80" spans="1:9" ht="15.75" customHeight="1">
       <c r="A80" s="84">
         <v>46020</v>
       </c>
@@ -14527,7 +14535,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="81" spans="1:9" ht="13.5" customHeight="1">
       <c r="A81" s="82">
         <v>46024</v>
       </c>
@@ -14552,7 +14560,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="82" spans="1:9" ht="15.75" customHeight="1">
       <c r="A82" s="84">
         <v>46024</v>
       </c>
@@ -14577,7 +14585,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="83" spans="1:9" ht="13.5" customHeight="1">
       <c r="A83" s="82">
         <v>46024</v>
       </c>
@@ -14602,7 +14610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="84" spans="1:9" ht="15.75" customHeight="1">
       <c r="A84" s="84">
         <v>46024</v>
       </c>
@@ -14627,7 +14635,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="85" spans="1:9" ht="13.5" customHeight="1">
       <c r="A85" s="82">
         <v>46027</v>
       </c>
@@ -14652,7 +14660,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="86" spans="1:9" ht="13.5" customHeight="1">
       <c r="A86" s="82">
         <v>46028</v>
       </c>
@@ -14677,7 +14685,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="87" spans="1:9" ht="15.75" customHeight="1">
       <c r="A87" s="84">
         <v>46029</v>
       </c>
@@ -14702,7 +14710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="88" spans="1:9" ht="13.5" customHeight="1">
       <c r="A88" s="82">
         <v>46032</v>
       </c>
@@ -14727,7 +14735,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="89" spans="1:9" ht="15.75" customHeight="1">
       <c r="A89" s="84">
         <v>46033</v>
       </c>
@@ -14752,7 +14760,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="90" spans="1:9" ht="13.5" customHeight="1">
       <c r="A90" s="82">
         <v>46033</v>
       </c>
@@ -14777,7 +14785,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="91" spans="1:9" ht="15.75" customHeight="1">
       <c r="A91" s="84">
         <v>46034</v>
       </c>
@@ -14802,7 +14810,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="92" spans="1:9" ht="27.75" customHeight="1">
       <c r="A92" s="82">
         <v>46034</v>
       </c>
@@ -14827,7 +14835,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="93" spans="1:9" ht="15.75" customHeight="1">
       <c r="A93" s="84">
         <v>46035</v>
       </c>
@@ -14852,7 +14860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="94" spans="1:9" ht="13.5" customHeight="1">
       <c r="A94" s="82">
         <v>46036</v>
       </c>
@@ -14877,7 +14885,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="95" spans="1:9" ht="15.75" customHeight="1">
       <c r="A95" s="84">
         <v>46038</v>
       </c>
@@ -14902,7 +14910,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="96" spans="1:9" ht="13.5" customHeight="1">
       <c r="A96" s="82">
         <v>46038</v>
       </c>
@@ -14927,7 +14935,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="97" spans="1:9" ht="15.75" customHeight="1">
       <c r="A97" s="84">
         <v>46039</v>
       </c>
@@ -14952,7 +14960,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="98" spans="1:9" ht="13.5" customHeight="1">
       <c r="A98" s="82">
         <v>46040</v>
       </c>
@@ -14977,7 +14985,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="99" spans="1:9" ht="15.75" customHeight="1">
       <c r="A99" s="84">
         <v>46041</v>
       </c>
@@ -15002,7 +15010,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="100" spans="1:9" ht="13.5" customHeight="1">
       <c r="A100" s="82">
         <v>46042</v>
       </c>
@@ -15027,7 +15035,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="101" spans="1:9" ht="15.75" customHeight="1">
       <c r="A101" s="84">
         <v>46043</v>
       </c>
@@ -15052,7 +15060,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="102" spans="1:9" ht="13.5" customHeight="1">
       <c r="A102" s="82">
         <v>46046</v>
       </c>
@@ -15077,7 +15085,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="103" spans="1:9" ht="13.5" customHeight="1">
       <c r="A103" s="84">
         <v>46048</v>
       </c>
@@ -15102,7 +15110,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="104" spans="1:9" ht="13.5" customHeight="1">
       <c r="A104" s="82">
         <v>46048</v>
       </c>
@@ -15127,7 +15135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="105" spans="1:9" ht="15.75" customHeight="1">
       <c r="A105" s="84">
         <v>46049</v>
       </c>
@@ -15152,7 +15160,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="106" spans="1:9" ht="13.5" customHeight="1">
       <c r="A106" s="82">
         <v>46049</v>
       </c>
@@ -15177,7 +15185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="107" spans="1:9" ht="15.75" customHeight="1">
       <c r="A107" s="84">
         <v>46049</v>
       </c>
@@ -15202,7 +15210,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="108" spans="1:9" ht="13.5" customHeight="1">
       <c r="A108" s="82">
         <v>46050</v>
       </c>
@@ -15227,7 +15235,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="109" spans="1:9" ht="15.75" customHeight="1">
       <c r="A109" s="84">
         <v>46051</v>
       </c>
@@ -15252,7 +15260,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="110" spans="1:9" ht="13.5" customHeight="1">
       <c r="A110" s="82">
         <v>46051</v>
       </c>
@@ -15277,7 +15285,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="111" spans="1:9" ht="15.75" customHeight="1">
       <c r="A111" s="84">
         <v>46051</v>
       </c>
@@ -15302,7 +15310,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="112" spans="1:9" ht="27.75" customHeight="1">
       <c r="A112" s="82">
         <v>46054</v>
       </c>
@@ -15327,7 +15335,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="113" spans="1:9" ht="15.75" customHeight="1">
       <c r="A113" s="84">
         <v>46054</v>
       </c>
@@ -15352,7 +15360,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="114" spans="1:9" ht="13.5" customHeight="1">
       <c r="A114" s="82">
         <v>46055</v>
       </c>
@@ -15377,7 +15385,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="115" spans="1:9" ht="15.75" customHeight="1">
       <c r="A115" s="84">
         <v>46055</v>
       </c>
@@ -15402,7 +15410,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="116" spans="1:9" ht="13.5" customHeight="1">
       <c r="A116" s="82">
         <v>46060</v>
       </c>
@@ -15427,7 +15435,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="117" spans="1:9" ht="15.75" customHeight="1">
       <c r="A117" s="84">
         <v>46062</v>
       </c>
@@ -15452,7 +15460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="118" spans="1:9" ht="13.5" customHeight="1">
       <c r="A118" s="82">
         <v>46065</v>
       </c>
@@ -15477,7 +15485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="119" spans="1:9" ht="15.75" customHeight="1">
       <c r="A119" s="84">
         <v>46055</v>
       </c>
@@ -15502,7 +15510,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="120" spans="1:9" ht="27.75" customHeight="1">
       <c r="A120" s="82">
         <v>46070</v>
       </c>
@@ -15527,7 +15535,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="121" spans="1:9" ht="15.75" customHeight="1">
       <c r="A121" s="84">
         <v>46073</v>
       </c>
@@ -15552,7 +15560,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="122" spans="1:9" ht="13.5" customHeight="1">
       <c r="A122" s="82">
         <v>46074</v>
       </c>
@@ -15577,7 +15585,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="123" spans="1:9" ht="15.75" customHeight="1">
       <c r="A123" s="84">
         <v>46075</v>
       </c>
@@ -15602,7 +15610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="124" spans="1:9" ht="13.5" customHeight="1">
       <c r="A124" s="82">
         <v>46075</v>
       </c>
@@ -15652,7 +15660,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="126" spans="1:9" ht="13.5" customHeight="1">
       <c r="A126" s="82">
         <v>46079</v>
       </c>
@@ -15677,7 +15685,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="127" spans="1:9" ht="13.5" customHeight="1">
       <c r="A127" s="84">
         <v>46090</v>
       </c>
@@ -15702,7 +15710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="128" spans="1:9" ht="13.5" customHeight="1">
       <c r="A128" s="82">
         <v>46090</v>
       </c>
@@ -15727,7 +15735,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="129" spans="1:9" ht="13.5" customHeight="1">
       <c r="A129" s="82">
         <v>46090</v>
       </c>
@@ -15752,7 +15760,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="130" spans="1:9" ht="15.75" customHeight="1">
       <c r="A130" s="84">
         <v>46091</v>
       </c>
@@ -15777,7 +15785,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="131" spans="1:9" ht="13.5" customHeight="1">
       <c r="A131" s="82">
         <v>46092</v>
       </c>
@@ -15802,7 +15810,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="132" spans="1:9" ht="15.75" customHeight="1">
       <c r="A132" s="84">
         <v>46092</v>
       </c>
@@ -15827,7 +15835,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="133" spans="1:9" ht="27.75" customHeight="1">
       <c r="A133" s="82">
         <v>46093</v>
       </c>
@@ -15852,7 +15860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="134" spans="1:9" ht="15.75" customHeight="1">
       <c r="A134" s="84">
         <v>46093</v>
       </c>
@@ -15877,7 +15885,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="135" spans="1:9" ht="13.5" customHeight="1">
       <c r="A135" s="82">
         <v>46097</v>
       </c>
@@ -15902,7 +15910,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="136" spans="1:9" ht="15.75" customHeight="1">
       <c r="A136" s="84">
         <v>46097</v>
       </c>
@@ -15927,7 +15935,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="137" spans="1:9" ht="13.5" customHeight="1">
       <c r="A137" s="82">
         <v>46100</v>
       </c>
@@ -15952,7 +15960,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="138" spans="1:9" ht="15.75" customHeight="1">
       <c r="A138" s="84">
         <v>46104</v>
       </c>
@@ -15977,7 +15985,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="139" spans="1:9" ht="27.75" customHeight="1">
       <c r="A139" s="82">
         <v>46105</v>
       </c>
@@ -16002,7 +16010,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="31.5" hidden="1" customHeight="1">
+    <row r="140" spans="1:9" ht="31.5" customHeight="1">
       <c r="A140" s="84">
         <v>46113</v>
       </c>
@@ -16027,7 +16035,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="141" spans="1:9" ht="13.5" customHeight="1">
       <c r="A141" s="82">
         <v>46118</v>
       </c>
@@ -16052,7 +16060,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="142" spans="1:9" ht="15.75" customHeight="1">
       <c r="A142" s="84">
         <v>46119</v>
       </c>
@@ -16077,7 +16085,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="143" spans="1:9" ht="13.5" customHeight="1">
       <c r="A143" s="82">
         <v>46120</v>
       </c>
@@ -16102,7 +16110,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="144" spans="1:9" ht="15.75" customHeight="1">
       <c r="A144" s="84">
         <v>46120</v>
       </c>
@@ -16127,7 +16135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="145" spans="1:9" ht="13.5" customHeight="1">
       <c r="A145" s="82">
         <v>46120</v>
       </c>
@@ -16152,7 +16160,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="31.5" hidden="1" customHeight="1">
+    <row r="146" spans="1:9" ht="31.5" customHeight="1">
       <c r="A146" s="84">
         <v>46122</v>
       </c>
@@ -16177,7 +16185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="147" spans="1:9" ht="13.5" customHeight="1">
       <c r="A147" s="82">
         <v>46122</v>
       </c>
@@ -16202,7 +16210,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="148" spans="1:9" ht="15.75" customHeight="1">
       <c r="A148" s="84">
         <v>46122</v>
       </c>
@@ -16252,7 +16260,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="150" spans="1:9" ht="15.75" customHeight="1">
       <c r="A150" s="84">
         <v>46125</v>
       </c>
@@ -16277,7 +16285,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="151" spans="1:9" ht="13.5" customHeight="1">
       <c r="A151" s="82">
         <v>46125</v>
       </c>
@@ -16302,7 +16310,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="152" spans="1:9" ht="15.75" customHeight="1">
       <c r="A152" s="84">
         <v>46125</v>
       </c>
@@ -16327,7 +16335,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="153" spans="1:9" ht="13.5" customHeight="1">
       <c r="A153" s="82">
         <v>46125</v>
       </c>
@@ -16352,7 +16360,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="154" spans="1:9" ht="15.75" customHeight="1">
       <c r="A154" s="84">
         <v>46126</v>
       </c>
@@ -16377,7 +16385,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="155" spans="1:9" ht="13.5" customHeight="1">
       <c r="A155" s="82">
         <v>46127</v>
       </c>
@@ -16402,7 +16410,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="156" spans="1:9" ht="15.75" customHeight="1">
       <c r="A156" s="84">
         <v>46129</v>
       </c>
@@ -16427,7 +16435,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="157" spans="1:9" ht="13.5" customHeight="1">
       <c r="A157" s="82">
         <v>46129</v>
       </c>
@@ -16452,7 +16460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="158" spans="1:9" ht="15.75" customHeight="1">
       <c r="A158" s="84">
         <v>46129</v>
       </c>
@@ -16477,7 +16485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="159" spans="1:9" ht="13.5" customHeight="1">
       <c r="A159" s="82">
         <v>46130</v>
       </c>
@@ -16502,7 +16510,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15.75" hidden="1" customHeight="1">
+    <row r="160" spans="1:9" ht="15.75" customHeight="1">
       <c r="A160" s="84">
         <v>46131</v>
       </c>
@@ -16527,7 +16535,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="161" spans="1:9" ht="13.5" customHeight="1">
       <c r="A161" s="82">
         <v>46132</v>
       </c>
@@ -16552,7 +16560,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="162" spans="1:9" ht="42" customHeight="1">
       <c r="A162" s="84">
         <v>46132</v>
       </c>
@@ -16577,7 +16585,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="163" spans="1:9" ht="13.5" customHeight="1">
       <c r="A163" s="82">
         <v>46133</v>
       </c>
@@ -16602,7 +16610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="164" spans="1:9" ht="13.5" customHeight="1">
       <c r="A164" s="84">
         <v>46133</v>
       </c>
@@ -16627,7 +16635,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="165" spans="1:9" ht="13.5" customHeight="1">
       <c r="A165" s="82">
         <v>46133</v>
       </c>
@@ -16652,7 +16660,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="166" spans="1:9" ht="13.5" customHeight="1">
       <c r="A166" s="84">
         <v>46134</v>
       </c>
@@ -16677,7 +16685,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="167" spans="1:9" ht="13.5" customHeight="1">
       <c r="A167" s="82">
         <v>46134</v>
       </c>
@@ -16702,7 +16710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="168" spans="1:9" ht="13.5" customHeight="1">
       <c r="A168" s="82">
         <v>46134</v>
       </c>
@@ -16727,7 +16735,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="169" spans="1:9" ht="13.5" customHeight="1">
       <c r="A169" s="84">
         <v>46134</v>
       </c>
@@ -16752,7 +16760,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="170" spans="1:9" ht="13.5" customHeight="1">
       <c r="A170" s="82">
         <v>46134</v>
       </c>
@@ -16777,7 +16785,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="171" spans="1:9" ht="13.5" customHeight="1">
       <c r="A171" s="84">
         <v>46136</v>
       </c>
@@ -16802,7 +16810,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="172" spans="1:9" ht="13.5" customHeight="1">
       <c r="A172" s="82">
         <v>46138</v>
       </c>
@@ -16827,7 +16835,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="173" spans="1:9" ht="13.5" customHeight="1">
       <c r="A173" s="84">
         <v>46138</v>
       </c>
@@ -16852,7 +16860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="174" spans="1:9" ht="13.5" customHeight="1">
       <c r="A174" s="82">
         <v>46139</v>
       </c>
@@ -16877,7 +16885,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="175" spans="1:9" ht="13.5" customHeight="1">
       <c r="A175" s="84">
         <v>46139</v>
       </c>
@@ -16902,7 +16910,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="176" spans="1:9" ht="13.5" customHeight="1">
       <c r="A176" s="82">
         <v>46139</v>
       </c>
@@ -16927,7 +16935,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="177" spans="1:9" ht="13.5" customHeight="1">
       <c r="A177" s="84">
         <v>46140</v>
       </c>
@@ -16952,7 +16960,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="178" spans="1:9" ht="13.5" customHeight="1">
       <c r="A178" s="82">
         <v>46140</v>
       </c>
@@ -16977,7 +16985,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="179" spans="1:9" ht="13.5" customHeight="1">
       <c r="A179" s="84">
         <v>46140</v>
       </c>
@@ -17002,7 +17010,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="180" spans="1:9" ht="13.5" customHeight="1">
       <c r="A180" s="82">
         <v>46140</v>
       </c>
@@ -17027,7 +17035,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="181" spans="1:9" ht="13.5" customHeight="1">
       <c r="A181" s="84">
         <v>46141</v>
       </c>
@@ -17052,7 +17060,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="182" spans="1:9" ht="13.5" customHeight="1">
       <c r="A182" s="82">
         <v>46141</v>
       </c>
@@ -17077,7 +17085,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="183" spans="1:9" ht="13.5" customHeight="1">
       <c r="A183" s="84">
         <v>46142</v>
       </c>
@@ -17102,7 +17110,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="184" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="184" spans="1:9" ht="13.5" customHeight="1">
       <c r="A184" s="82">
         <v>46142</v>
       </c>
@@ -17127,7 +17135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="185" spans="1:9" ht="13.5" customHeight="1">
       <c r="A185" s="84">
         <v>46142</v>
       </c>
@@ -17152,7 +17160,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="186" spans="1:9" ht="13.5" customHeight="1">
       <c r="A186" s="84">
         <v>46144</v>
       </c>
@@ -17202,7 +17210,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="188" spans="1:9" ht="13.5" customHeight="1">
       <c r="A188" s="84">
         <v>46145</v>
       </c>
@@ -17227,7 +17235,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="189" spans="1:9" ht="13.5" customHeight="1">
       <c r="A189" s="82">
         <v>46145</v>
       </c>
@@ -17252,7 +17260,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="190" spans="1:9" ht="13.5" customHeight="1">
       <c r="A190" s="84">
         <v>46145</v>
       </c>
@@ -17277,7 +17285,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="191" spans="1:9" ht="42" customHeight="1">
       <c r="A191" s="82">
         <v>46151</v>
       </c>
@@ -17302,7 +17310,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="192" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="192" spans="1:9" ht="27.75" customHeight="1">
       <c r="A192" s="84">
         <v>46152</v>
       </c>
@@ -17327,7 +17335,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="193" spans="1:9" ht="42" customHeight="1">
       <c r="A193" s="82">
         <v>46152</v>
       </c>
@@ -17352,7 +17360,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="194" spans="1:9" ht="27.75" customHeight="1">
       <c r="A194" s="84">
         <v>46151</v>
       </c>
@@ -17377,7 +17385,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="195" spans="1:9" ht="42" customHeight="1">
       <c r="A195" s="82">
         <v>46155</v>
       </c>
@@ -17402,7 +17410,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="196" spans="1:9" ht="42" customHeight="1">
       <c r="A196" s="84">
         <v>46155</v>
       </c>
@@ -17427,7 +17435,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="197" spans="1:9" ht="42" customHeight="1">
       <c r="A197" s="82">
         <v>46155</v>
       </c>
@@ -17452,7 +17460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="42" hidden="1" customHeight="1">
+    <row r="198" spans="1:9" ht="42" customHeight="1">
       <c r="A198" s="84">
         <v>46168</v>
       </c>
@@ -17477,7 +17485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="199" spans="1:9" ht="13.5" customHeight="1">
       <c r="A199" s="82">
         <v>46172</v>
       </c>
@@ -17502,7 +17510,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="200" spans="1:9" ht="27.75" customHeight="1">
       <c r="A200" s="84">
         <v>46173</v>
       </c>
@@ -17527,7 +17535,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="201" spans="1:9" ht="27.75" customHeight="1">
       <c r="A201" s="82">
         <v>46173</v>
       </c>
@@ -17552,7 +17560,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="202" spans="1:9" ht="13.5" customHeight="1">
       <c r="A202" s="84">
         <v>46173</v>
       </c>
@@ -17577,7 +17585,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="203" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="203" spans="1:9" ht="13.5" customHeight="1">
       <c r="A203" s="82">
         <v>46173</v>
       </c>
@@ -17602,7 +17610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="204" spans="1:9" ht="13.5" customHeight="1">
       <c r="A204" s="84">
         <v>46175</v>
       </c>
@@ -17627,7 +17635,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="205" spans="1:9" ht="13.5" customHeight="1">
       <c r="A205" s="82">
         <v>46175</v>
       </c>
@@ -17652,7 +17660,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="206" spans="1:9" ht="13.5" customHeight="1">
       <c r="A206" s="84">
         <v>46175</v>
       </c>
@@ -17677,7 +17685,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="207" spans="1:9" ht="13.5" customHeight="1">
       <c r="A207" s="82">
         <v>46175</v>
       </c>
@@ -17702,7 +17710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="208" spans="1:9" ht="13.5" customHeight="1">
       <c r="A208" s="84">
         <v>46175</v>
       </c>
@@ -17727,7 +17735,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="209" spans="1:9" ht="13.5" customHeight="1">
       <c r="A209" s="82">
         <v>46176</v>
       </c>
@@ -17752,7 +17760,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="210" spans="1:9" ht="27.75" customHeight="1">
       <c r="A210" s="84">
         <v>46176</v>
       </c>
@@ -17777,7 +17785,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="211" spans="1:9" ht="13.5" customHeight="1">
       <c r="A211" s="82">
         <v>46176</v>
       </c>
@@ -17802,7 +17810,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="14" hidden="1">
+    <row r="212" spans="1:9" ht="14">
       <c r="A212" s="84">
         <v>46176</v>
       </c>
@@ -17827,7 +17835,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="213" spans="1:9" ht="13.5" customHeight="1">
       <c r="A213" s="82">
         <v>46176</v>
       </c>
@@ -17877,7 +17885,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="215" spans="1:9" ht="13.5" customHeight="1">
       <c r="A215" s="82">
         <v>46187</v>
       </c>
@@ -17902,7 +17910,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="55.5" hidden="1" customHeight="1">
+    <row r="216" spans="1:9" ht="55.5" customHeight="1">
       <c r="A216" s="84">
         <v>46188</v>
       </c>
@@ -17927,7 +17935,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="217" spans="1:9" ht="13.5" customHeight="1">
       <c r="A217" s="84">
         <v>46191</v>
       </c>
@@ -17952,7 +17960,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="218" spans="1:9" ht="13.5" customHeight="1">
       <c r="A218" s="82">
         <v>46191</v>
       </c>
@@ -17977,7 +17985,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="219" spans="1:9" ht="13.5" customHeight="1">
       <c r="A219" s="84">
         <v>46191</v>
       </c>
@@ -18002,7 +18010,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="220" spans="1:9" ht="13.5" customHeight="1">
       <c r="A220" s="82">
         <v>46191</v>
       </c>
@@ -18027,7 +18035,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="221" spans="1:9" ht="13.5" customHeight="1">
       <c r="A221" s="84">
         <v>46191</v>
       </c>
@@ -18052,7 +18060,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="222" spans="1:9" ht="13.5" customHeight="1">
       <c r="A222" s="82">
         <v>46191</v>
       </c>
@@ -18077,7 +18085,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="223" spans="1:9" ht="13.5" customHeight="1">
       <c r="A223" s="84">
         <v>46191</v>
       </c>
@@ -18102,7 +18110,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="224" spans="1:9" ht="13.5" customHeight="1">
       <c r="A224" s="82">
         <v>46192</v>
       </c>
@@ -18127,7 +18135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="225" spans="1:9" ht="13.5" customHeight="1">
       <c r="A225" s="84">
         <v>46192</v>
       </c>
@@ -18152,7 +18160,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="226" spans="1:9" ht="13.5" customHeight="1">
       <c r="A226" s="82">
         <v>46192</v>
       </c>
@@ -18177,7 +18185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="227" spans="1:9" ht="13.5" customHeight="1">
       <c r="A227" s="84">
         <v>46192</v>
       </c>
@@ -18202,7 +18210,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="228" spans="1:9" ht="13.5" customHeight="1">
       <c r="A228" s="82">
         <v>46193</v>
       </c>
@@ -18227,7 +18235,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="229" spans="1:9" ht="13.5" customHeight="1">
       <c r="A229" s="84">
         <v>46193</v>
       </c>
@@ -18252,7 +18260,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="230" spans="1:9" ht="13.5" customHeight="1">
       <c r="A230" s="82">
         <v>46193</v>
       </c>
@@ -18277,7 +18285,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="231" spans="1:9" ht="13.5" customHeight="1">
       <c r="A231" s="84">
         <v>46193</v>
       </c>
@@ -18302,7 +18310,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="232" spans="1:9" ht="13.5" customHeight="1">
       <c r="A232" s="82">
         <v>46193</v>
       </c>
@@ -18327,7 +18335,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="233" spans="1:9" ht="13.5" customHeight="1">
       <c r="A233" s="84">
         <v>46193</v>
       </c>
@@ -18377,7 +18385,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="235" spans="1:9" ht="13.5" customHeight="1">
       <c r="A235" s="84">
         <v>46194</v>
       </c>
@@ -18402,7 +18410,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="236" spans="1:9" ht="27.75" customHeight="1">
       <c r="A236" s="82">
         <v>46194</v>
       </c>
@@ -18427,7 +18435,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="237" spans="1:9" ht="13.5" customHeight="1">
       <c r="A237" s="84">
         <v>46196</v>
       </c>
@@ -18452,7 +18460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="238" spans="1:9" ht="13.5" customHeight="1">
       <c r="A238" s="82">
         <v>46196</v>
       </c>
@@ -18477,7 +18485,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="239" spans="1:9" ht="13.5" customHeight="1">
       <c r="A239" s="84">
         <v>46196</v>
       </c>
@@ -18502,7 +18510,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="27.75" hidden="1" customHeight="1">
+    <row r="240" spans="1:9" ht="27.75" customHeight="1">
       <c r="A240" s="82">
         <v>46196</v>
       </c>
@@ -18527,7 +18535,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="241" spans="1:9" ht="13.5" customHeight="1">
       <c r="A241" s="84">
         <v>46197</v>
       </c>
@@ -18552,7 +18560,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="242" spans="1:9" ht="13.5" customHeight="1">
       <c r="A242" s="82">
         <v>46197</v>
       </c>
@@ -18577,7 +18585,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="243" spans="1:9" ht="13.5" customHeight="1">
       <c r="A243" s="84">
         <v>46197</v>
       </c>
@@ -18602,7 +18610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="244" spans="1:9" ht="13.5" customHeight="1">
       <c r="A244" s="82">
         <v>46197</v>
       </c>
@@ -18627,7 +18635,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="245" spans="1:9" ht="13.5" customHeight="1">
       <c r="A245" s="84">
         <v>46198</v>
       </c>
@@ -18652,7 +18660,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="246" spans="1:9" ht="13.5" customHeight="1">
       <c r="A246" s="82">
         <v>46199</v>
       </c>
@@ -18677,7 +18685,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="247" spans="1:9" ht="13.5" customHeight="1">
       <c r="A247" s="84">
         <v>46199</v>
       </c>
@@ -18702,7 +18710,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="13.5" hidden="1" customHeight="1">
+    <row r="248" spans="1:9" ht="13.5" customHeight="1">
       <c r="A248" s="82">
         <v>46199</v>
       </c>
@@ -18752,7 +18760,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="14" hidden="1">
+    <row r="250" spans="1:9" ht="14">
       <c r="A250" s="82">
         <v>46200</v>
       </c>
@@ -18773,7 +18781,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="14" hidden="1">
+    <row r="251" spans="1:9" ht="14">
       <c r="A251" s="84">
         <v>46201</v>
       </c>
@@ -18798,7 +18806,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="14" hidden="1">
+    <row r="252" spans="1:9" ht="14">
       <c r="A252" s="82">
         <v>46201</v>
       </c>
@@ -18823,7 +18831,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="14" hidden="1">
+    <row r="253" spans="1:9" ht="14">
       <c r="A253" s="84">
         <v>46201</v>
       </c>
@@ -18848,7 +18856,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="14" hidden="1">
+    <row r="254" spans="1:9" ht="14">
       <c r="A254" s="82">
         <v>46201</v>
       </c>
@@ -18873,7 +18881,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="14" hidden="1">
+    <row r="255" spans="1:9" ht="14">
       <c r="A255" s="84">
         <v>46201</v>
       </c>
@@ -18898,7 +18906,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="14" hidden="1">
+    <row r="256" spans="1:9" ht="14">
       <c r="A256" s="82">
         <v>46203</v>
       </c>
@@ -18923,7 +18931,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="14" hidden="1">
+    <row r="257" spans="1:9" ht="14">
       <c r="A257" s="84">
         <v>46204</v>
       </c>
@@ -18948,7 +18956,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="14" hidden="1">
+    <row r="258" spans="1:9" ht="14">
       <c r="A258" s="82">
         <v>46205</v>
       </c>
@@ -18973,7 +18981,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="14" hidden="1">
+    <row r="259" spans="1:9" ht="14">
       <c r="A259" s="84">
         <v>46205</v>
       </c>
@@ -18998,7 +19006,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="14" hidden="1">
+    <row r="260" spans="1:9" ht="14">
       <c r="A260" s="82">
         <v>46205</v>
       </c>
@@ -19023,7 +19031,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="14" hidden="1">
+    <row r="261" spans="1:9" ht="14">
       <c r="A261" s="84">
         <v>46205</v>
       </c>
@@ -19048,7 +19056,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="14" hidden="1">
+    <row r="262" spans="1:9" ht="14">
       <c r="A262" s="82">
         <v>46206</v>
       </c>
@@ -19073,7 +19081,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="14" hidden="1">
+    <row r="263" spans="1:9" ht="14">
       <c r="A263" s="84">
         <v>46206</v>
       </c>
@@ -19098,7 +19106,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="42" hidden="1">
+    <row r="264" spans="1:9" ht="42">
       <c r="A264" s="82">
         <v>46206</v>
       </c>
@@ -19123,7 +19131,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="14" hidden="1">
+    <row r="265" spans="1:9" ht="14">
       <c r="A265" s="84">
         <v>46206</v>
       </c>
@@ -19148,7 +19156,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="14" hidden="1">
+    <row r="266" spans="1:9" ht="14">
       <c r="A266" s="82">
         <v>46206</v>
       </c>
@@ -19173,7 +19181,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="14" hidden="1">
+    <row r="267" spans="1:9" ht="14">
       <c r="A267" s="84">
         <v>46207</v>
       </c>
@@ -19198,12 +19206,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="42" hidden="1">
+    <row r="268" spans="1:9" ht="42">
       <c r="A268" s="82">
         <v>46208</v>
       </c>
       <c r="B268" s="44" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C268" s="83">
         <v>2350</v>
@@ -19213,13 +19221,13 @@
       <c r="F268" s="44"/>
       <c r="G268" s="44"/>
       <c r="H268" s="44" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="I268" s="44" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="14" hidden="1">
+    <row r="269" spans="1:9" ht="14">
       <c r="A269" s="84">
         <v>46209</v>
       </c>
@@ -19244,12 +19252,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="14" hidden="1">
+    <row r="270" spans="1:9" ht="14">
       <c r="A270" s="82">
         <v>46210</v>
       </c>
       <c r="B270" s="44" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C270" s="83">
         <v>3200</v>
@@ -19269,7 +19277,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="14" hidden="1">
+    <row r="271" spans="1:9" ht="14">
       <c r="A271" s="84">
         <v>46211</v>
       </c>
@@ -19294,7 +19302,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="14" hidden="1">
+    <row r="272" spans="1:9" ht="14">
       <c r="A272" s="82">
         <v>46215</v>
       </c>
@@ -19319,7 +19327,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="14" hidden="1">
+    <row r="273" spans="1:9" ht="14">
       <c r="A273" s="84">
         <v>46215</v>
       </c>
@@ -19344,7 +19352,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="14" hidden="1">
+    <row r="274" spans="1:9" ht="14">
       <c r="A274" s="82">
         <v>46215</v>
       </c>
@@ -19369,7 +19377,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="14" hidden="1">
+    <row r="275" spans="1:9" ht="14">
       <c r="A275" s="84">
         <v>46216</v>
       </c>
@@ -19394,7 +19402,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="14" hidden="1">
+    <row r="276" spans="1:9" ht="14">
       <c r="A276" s="82">
         <v>46216</v>
       </c>
@@ -19419,7 +19427,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="14" hidden="1">
+    <row r="277" spans="1:9" ht="14">
       <c r="A277" s="84">
         <v>46219</v>
       </c>
@@ -19444,7 +19452,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="14" hidden="1">
+    <row r="278" spans="1:9" ht="14">
       <c r="A278" s="82">
         <v>46219</v>
       </c>
@@ -19469,7 +19477,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="14" hidden="1">
+    <row r="279" spans="1:9" ht="14">
       <c r="A279" s="84">
         <v>46219</v>
       </c>
@@ -19494,7 +19502,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="14" hidden="1">
+    <row r="280" spans="1:9" ht="14">
       <c r="A280" s="82">
         <v>46219</v>
       </c>
@@ -19524,7 +19532,7 @@
         <v>46219</v>
       </c>
       <c r="B281" s="45" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="C281" s="85">
         <v>3600</v>
@@ -19538,13 +19546,13 @@
       <c r="F281" s="46"/>
       <c r="G281" s="46"/>
       <c r="H281" s="46" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="I281" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="14" hidden="1">
+    <row r="282" spans="1:9" ht="14">
       <c r="A282" s="82">
         <v>46220</v>
       </c>
@@ -19569,7 +19577,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="14" hidden="1">
+    <row r="283" spans="1:9" ht="14">
       <c r="A283" s="84">
         <v>46221</v>
       </c>
@@ -19594,7 +19602,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="14" hidden="1">
+    <row r="284" spans="1:9" ht="14">
       <c r="A284" s="82">
         <v>46222</v>
       </c>
@@ -19619,7 +19627,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="14" hidden="1">
+    <row r="285" spans="1:9" ht="14">
       <c r="A285" s="84">
         <v>46222</v>
       </c>
@@ -19644,7 +19652,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="14" hidden="1">
+    <row r="286" spans="1:9" ht="14">
       <c r="A286" s="82">
         <v>46222</v>
       </c>
@@ -19669,7 +19677,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="14" hidden="1">
+    <row r="287" spans="1:9" ht="14">
       <c r="A287" s="84">
         <v>46222</v>
       </c>
@@ -19694,7 +19702,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="14" hidden="1">
+    <row r="288" spans="1:9" ht="14">
       <c r="A288" s="82">
         <v>46223</v>
       </c>
@@ -19719,7 +19727,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="14" hidden="1">
+    <row r="289" spans="1:9" ht="14">
       <c r="A289" s="84">
         <v>46224</v>
       </c>
@@ -19744,7 +19752,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="14" hidden="1">
+    <row r="290" spans="1:9" ht="14">
       <c r="A290" s="82">
         <v>46224</v>
       </c>
@@ -19769,7 +19777,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="14" hidden="1">
+    <row r="291" spans="1:9" ht="14">
       <c r="A291" s="82">
         <v>46228</v>
       </c>
@@ -19794,7 +19802,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="56" hidden="1">
+    <row r="292" spans="1:9" ht="56">
       <c r="A292" s="84">
         <v>46229</v>
       </c>
@@ -19809,13 +19817,13 @@
       <c r="F292" s="46"/>
       <c r="G292" s="46"/>
       <c r="H292" s="46" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="I292" s="45" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="28" hidden="1">
+    <row r="293" spans="1:9" ht="28">
       <c r="A293" s="82">
         <v>46229</v>
       </c>
@@ -19830,13 +19838,13 @@
       <c r="F293" s="44"/>
       <c r="G293" s="44"/>
       <c r="H293" s="44" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="I293" s="44" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="14" hidden="1">
+    <row r="294" spans="1:9" ht="14">
       <c r="A294" s="84">
         <v>46229</v>
       </c>
@@ -19855,13 +19863,13 @@
       <c r="F294" s="46"/>
       <c r="G294" s="46"/>
       <c r="H294" s="46" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="I294" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="28" hidden="1">
+    <row r="295" spans="1:9" ht="28">
       <c r="A295" s="82">
         <v>46229</v>
       </c>
@@ -19872,7 +19880,7 @@
         <v>3700</v>
       </c>
       <c r="D295" s="44" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="E295" s="44" t="s">
         <v>49</v>
@@ -19880,13 +19888,13 @@
       <c r="F295" s="44"/>
       <c r="G295" s="44"/>
       <c r="H295" s="44" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="I295" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="14" hidden="1">
+    <row r="296" spans="1:9" ht="14">
       <c r="A296" s="84">
         <v>46235</v>
       </c>
@@ -19911,12 +19919,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="14" hidden="1">
+    <row r="297" spans="1:9" ht="14">
       <c r="A297" s="82">
         <v>46236</v>
       </c>
       <c r="B297" s="44" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C297" s="83">
         <v>6900</v>
@@ -19930,13 +19938,13 @@
       <c r="F297" s="44"/>
       <c r="G297" s="44"/>
       <c r="H297" s="44" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="I297" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="14" hidden="1">
+    <row r="298" spans="1:9" ht="14">
       <c r="A298" s="84">
         <v>46236</v>
       </c>
@@ -19961,7 +19969,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="14" hidden="1">
+    <row r="299" spans="1:9" ht="14">
       <c r="A299" s="82">
         <v>46236</v>
       </c>
@@ -19986,7 +19994,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="14" hidden="1">
+    <row r="300" spans="1:9" ht="14">
       <c r="A300" s="84">
         <v>46238</v>
       </c>
@@ -20011,12 +20019,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="14" hidden="1">
+    <row r="301" spans="1:9" ht="14">
       <c r="A301" s="82">
         <v>46238</v>
       </c>
       <c r="B301" s="44" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C301" s="83">
         <v>12650</v>
@@ -20030,13 +20038,13 @@
       <c r="F301" s="44"/>
       <c r="G301" s="44"/>
       <c r="H301" s="44" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="I301" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="14" hidden="1">
+    <row r="302" spans="1:9" ht="14">
       <c r="A302" s="84">
         <v>46240</v>
       </c>
@@ -20057,7 +20065,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="42" hidden="1">
+    <row r="303" spans="1:9" ht="42">
       <c r="A303" s="82">
         <v>46241</v>
       </c>
@@ -20072,13 +20080,13 @@
       <c r="F303" s="44"/>
       <c r="G303" s="44"/>
       <c r="H303" s="44" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="I303" s="44" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="14" hidden="1">
+    <row r="304" spans="1:9" ht="14">
       <c r="A304" s="84">
         <v>46243</v>
       </c>
@@ -20099,7 +20107,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="14" hidden="1">
+    <row r="305" spans="1:9" ht="14">
       <c r="A305" s="82">
         <v>46243</v>
       </c>
@@ -20124,7 +20132,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="14" hidden="1">
+    <row r="306" spans="1:9" ht="14">
       <c r="A306" s="84">
         <v>46243</v>
       </c>
@@ -20149,12 +20157,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="14" hidden="1">
+    <row r="307" spans="1:9" ht="14">
       <c r="A307" s="82">
         <v>46243</v>
       </c>
       <c r="B307" s="44" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C307" s="83">
         <v>5750</v>
@@ -20168,18 +20176,18 @@
       <c r="F307" s="44"/>
       <c r="G307" s="44"/>
       <c r="H307" s="44" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="I307" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="14" hidden="1">
+    <row r="308" spans="1:9" ht="14">
       <c r="A308" s="82">
         <v>46248</v>
       </c>
       <c r="B308" s="44" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C308" s="83">
         <v>1380</v>
@@ -20193,18 +20201,18 @@
       <c r="F308" s="44"/>
       <c r="G308" s="44"/>
       <c r="H308" s="44" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="I308" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="309" spans="1:9" ht="14" hidden="1">
+    <row r="309" spans="1:9" ht="14">
       <c r="A309" s="84">
         <v>46248</v>
       </c>
       <c r="B309" s="45" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C309" s="85">
         <v>1380</v>
@@ -20218,13 +20226,13 @@
       <c r="F309" s="46"/>
       <c r="G309" s="46"/>
       <c r="H309" s="46" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="I309" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="310" spans="1:9" ht="14" hidden="1">
+    <row r="310" spans="1:9" ht="14">
       <c r="A310" s="82">
         <v>46250</v>
       </c>
@@ -20243,13 +20251,13 @@
       <c r="F310" s="44"/>
       <c r="G310" s="44"/>
       <c r="H310" s="44" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="I310" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="311" spans="1:9" ht="14" hidden="1">
+    <row r="311" spans="1:9" ht="14">
       <c r="A311" s="84">
         <v>46250</v>
       </c>
@@ -20268,18 +20276,18 @@
       <c r="F311" s="46"/>
       <c r="G311" s="46"/>
       <c r="H311" s="46" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="I311" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="312" spans="1:9" ht="14" hidden="1">
+    <row r="312" spans="1:9" ht="14">
       <c r="A312" s="82">
         <v>46250</v>
       </c>
       <c r="B312" s="44" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C312" s="83">
         <v>2250</v>
@@ -20293,18 +20301,18 @@
       <c r="F312" s="44"/>
       <c r="G312" s="44"/>
       <c r="H312" s="44" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="I312" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="313" spans="1:9" ht="14" hidden="1">
+    <row r="313" spans="1:9" ht="14">
       <c r="A313" s="84">
         <v>46252</v>
       </c>
       <c r="B313" s="45" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C313" s="85">
         <v>5750</v>
@@ -20318,18 +20326,18 @@
       <c r="F313" s="46"/>
       <c r="G313" s="46"/>
       <c r="H313" s="46" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="I313" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="314" spans="1:9" ht="14" hidden="1">
+    <row r="314" spans="1:9" ht="14">
       <c r="A314" s="82">
         <v>46252</v>
       </c>
       <c r="B314" s="44" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="C314" s="83">
         <v>1380</v>
@@ -20343,18 +20351,18 @@
       <c r="F314" s="44"/>
       <c r="G314" s="44"/>
       <c r="H314" s="44" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="I314" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="315" spans="1:9" ht="14" hidden="1">
+    <row r="315" spans="1:9" ht="14">
       <c r="A315" s="84">
         <v>46252</v>
       </c>
       <c r="B315" s="45" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C315" s="85">
         <v>5750</v>
@@ -20368,18 +20376,18 @@
       <c r="F315" s="46"/>
       <c r="G315" s="46"/>
       <c r="H315" s="46" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="I315" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="316" spans="1:9" ht="14" hidden="1">
+    <row r="316" spans="1:9" ht="14">
       <c r="A316" s="82">
         <v>46252</v>
       </c>
       <c r="B316" s="44" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="C316" s="83">
         <v>1380</v>
@@ -20389,18 +20397,18 @@
       <c r="F316" s="44"/>
       <c r="G316" s="44"/>
       <c r="H316" s="44" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="I316" s="44" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="317" spans="1:9" ht="14" hidden="1">
+    <row r="317" spans="1:9" ht="14">
       <c r="A317" s="84">
         <v>46252</v>
       </c>
       <c r="B317" s="45" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="C317" s="85">
         <v>1250</v>
@@ -20414,18 +20422,18 @@
       <c r="F317" s="46"/>
       <c r="G317" s="46"/>
       <c r="H317" s="46" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="I317" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="318" spans="1:9" ht="14" hidden="1">
+    <row r="318" spans="1:9" ht="14">
       <c r="A318" s="82">
         <v>46257</v>
       </c>
       <c r="B318" s="44" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C318" s="83">
         <v>1780</v>
@@ -20439,13 +20447,13 @@
       <c r="F318" s="44"/>
       <c r="G318" s="44"/>
       <c r="H318" s="44" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="I318" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="319" spans="1:9" ht="14" hidden="1">
+    <row r="319" spans="1:9" ht="14">
       <c r="A319" s="84">
         <v>46257</v>
       </c>
@@ -20464,13 +20472,13 @@
       <c r="F319" s="46"/>
       <c r="G319" s="46"/>
       <c r="H319" s="46" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="I319" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="320" spans="1:9" ht="14" hidden="1">
+    <row r="320" spans="1:9" ht="14">
       <c r="A320" s="82">
         <v>46257</v>
       </c>
@@ -20489,18 +20497,18 @@
       <c r="F320" s="44"/>
       <c r="G320" s="44"/>
       <c r="H320" s="44" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="I320" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="321" spans="1:9" ht="14" hidden="1">
+    <row r="321" spans="1:9" ht="14">
       <c r="A321" s="84">
         <v>46257</v>
       </c>
       <c r="B321" s="45" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="C321" s="85">
         <v>1500</v>
@@ -20514,18 +20522,18 @@
       <c r="F321" s="46"/>
       <c r="G321" s="46"/>
       <c r="H321" s="46" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="I321" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="322" spans="1:9" ht="14" hidden="1">
+    <row r="322" spans="1:9" ht="14">
       <c r="A322" s="82">
         <v>46258</v>
       </c>
       <c r="B322" s="44" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="C322" s="83">
         <v>1250</v>
@@ -20539,18 +20547,18 @@
       <c r="F322" s="44"/>
       <c r="G322" s="44"/>
       <c r="H322" s="44" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="I322" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="323" spans="1:9" ht="14" hidden="1">
+    <row r="323" spans="1:9" ht="14">
       <c r="A323" s="84">
         <v>46263</v>
       </c>
       <c r="B323" s="45" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C323" s="85">
         <v>1380</v>
@@ -20564,18 +20572,18 @@
       <c r="F323" s="46"/>
       <c r="G323" s="46"/>
       <c r="H323" s="46" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="I323" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="324" spans="1:9" ht="14" hidden="1">
+    <row r="324" spans="1:9" ht="14">
       <c r="A324" s="82">
         <v>46263</v>
       </c>
       <c r="B324" s="44" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="C324" s="83">
         <v>1380</v>
@@ -20589,18 +20597,18 @@
       <c r="F324" s="44"/>
       <c r="G324" s="44"/>
       <c r="H324" s="44" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="I324" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="325" spans="1:9" ht="14" hidden="1">
+    <row r="325" spans="1:9" ht="14">
       <c r="A325" s="84">
         <v>46263</v>
       </c>
       <c r="B325" s="45" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C325" s="85">
         <v>2500</v>
@@ -20614,31 +20622,61 @@
       <c r="F325" s="46"/>
       <c r="G325" s="46"/>
       <c r="H325" s="46" t="s">
-        <v>1358</v>
-      </c>
-      <c r="I325" s="45"/>
-    </row>
-    <row r="326" spans="1:9">
-      <c r="A326" s="82"/>
-      <c r="B326" s="44"/>
-      <c r="C326" s="83"/>
-      <c r="D326" s="44"/>
-      <c r="E326" s="44"/>
+        <v>1368</v>
+      </c>
+      <c r="I325" s="45" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="326" spans="1:9" ht="14">
+      <c r="A326" s="82">
+        <v>46257</v>
+      </c>
+      <c r="B326" s="44" t="s">
+        <v>226</v>
+      </c>
+      <c r="C326" s="83">
+        <v>750</v>
+      </c>
+      <c r="D326" s="44" t="s">
+        <v>150</v>
+      </c>
+      <c r="E326" s="44" t="s">
+        <v>49</v>
+      </c>
       <c r="F326" s="44"/>
       <c r="G326" s="44"/>
-      <c r="H326" s="44"/>
-      <c r="I326" s="44"/>
-    </row>
-    <row r="327" spans="1:9">
-      <c r="A327" s="84"/>
-      <c r="B327" s="45"/>
-      <c r="C327" s="85"/>
-      <c r="D327" s="45"/>
-      <c r="E327" s="45"/>
+      <c r="H326" s="44" t="s">
+        <v>1367</v>
+      </c>
+      <c r="I326" s="44" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="327" spans="1:9" ht="14">
+      <c r="A327" s="84">
+        <v>46257</v>
+      </c>
+      <c r="B327" s="45" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C327" s="85">
+        <v>750</v>
+      </c>
+      <c r="D327" s="45" t="s">
+        <v>150</v>
+      </c>
+      <c r="E327" s="45" t="s">
+        <v>49</v>
+      </c>
       <c r="F327" s="46"/>
       <c r="G327" s="46"/>
-      <c r="H327" s="46"/>
-      <c r="I327" s="45"/>
+      <c r="H327" s="46" t="s">
+        <v>1370</v>
+      </c>
+      <c r="I327" s="45" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="328" spans="1:9">
       <c r="A328" s="82"/>
@@ -20652,16 +20690,7 @@
       <c r="I328" s="44"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I326" xr:uid="{00000000-0009-0000-0000-000004000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Asha Latha"/>
-        <filter val="Latha"/>
-        <filter val="Latha Ammayi"/>
-        <filter val="Latha Suresh (Malappuram)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I326" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1257" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -33622,7 +33651,7 @@
         <v>606</v>
       </c>
       <c r="L166" s="52" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="M166" s="52"/>
       <c r="N166" s="52" t="s">
@@ -33630,7 +33659,7 @@
       </c>
       <c r="O166" s="52"/>
       <c r="P166" s="52" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="Q166" s="52"/>
       <c r="R166" s="52"/>
@@ -34098,7 +34127,7 @@
         <v>2793</v>
       </c>
       <c r="L175" s="55" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="M175" s="55"/>
       <c r="N175" s="55" t="s">
@@ -34106,7 +34135,7 @@
       </c>
       <c r="O175" s="55"/>
       <c r="P175" s="55" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="Q175" s="55"/>
       <c r="R175" s="55"/>
@@ -34418,7 +34447,7 @@
         <v>1019</v>
       </c>
       <c r="L181" s="55" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="M181" s="55"/>
       <c r="N181" s="55" t="s">
@@ -34731,7 +34760,7 @@
         <v>891</v>
       </c>
       <c r="L187" s="55" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="M187" s="55"/>
       <c r="N187" s="55" t="s">
@@ -34835,7 +34864,7 @@
         <v>891</v>
       </c>
       <c r="L189" s="55" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="M189" s="55"/>
       <c r="N189" s="55" t="s">
@@ -34843,7 +34872,7 @@
       </c>
       <c r="O189" s="55"/>
       <c r="P189" s="55" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="Q189" s="55"/>
       <c r="R189" s="55"/>
@@ -35052,7 +35081,7 @@
         <v>982</v>
       </c>
       <c r="B194" s="52" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="C194" s="52" t="s">
         <v>95</v>
@@ -35086,14 +35115,14 @@
         <v>5530</v>
       </c>
       <c r="L194" s="52" t="s">
-        <v>1361</v>
+        <v>1359</v>
       </c>
       <c r="M194" s="52"/>
       <c r="N194" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P194" s="47" t="s">
-        <v>1362</v>
+        <v>1360</v>
       </c>
       <c r="S194" s="47"/>
       <c r="T194" s="47"/>
@@ -35337,14 +35366,14 @@
         <v>1732</v>
       </c>
       <c r="L199" s="52" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="M199" s="52"/>
       <c r="N199" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="47" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="S199" s="47"/>
       <c r="T199" s="47"/>
@@ -35592,14 +35621,14 @@
         <v>761</v>
       </c>
       <c r="L204" s="55" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="M204" s="55"/>
       <c r="N204" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="47" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="S204" s="47"/>
       <c r="T204" s="47"/>
@@ -35745,14 +35774,14 @@
         <v>2346</v>
       </c>
       <c r="L207" s="52" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="M207" s="52"/>
       <c r="N207" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P207" s="47" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="S207" s="47"/>
       <c r="T207" s="47"/>
@@ -35896,7 +35925,7 @@
         <v>0</v>
       </c>
       <c r="L210" s="55" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="M210" s="55"/>
       <c r="N210" s="47" t="s">
@@ -35947,7 +35976,7 @@
         <v>0</v>
       </c>
       <c r="L211" s="52" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="M211" s="52"/>
       <c r="N211" s="47" t="s">
@@ -35995,14 +36024,14 @@
         <v>2220</v>
       </c>
       <c r="L212" s="55" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="M212" s="55"/>
       <c r="N212" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P212" s="47" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="S212" s="47"/>
       <c r="T212" s="47"/>
@@ -36046,7 +36075,7 @@
         <v>3340</v>
       </c>
       <c r="L213" s="52" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="M213" s="52"/>
       <c r="N213" s="47" t="s">
@@ -36650,14 +36679,14 @@
         <v>940</v>
       </c>
       <c r="L225" s="52" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="M225" s="52"/>
       <c r="N225" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P225" s="86" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="S225" s="47"/>
       <c r="T225" s="47"/>
@@ -36801,14 +36830,14 @@
         <v>2775</v>
       </c>
       <c r="L228" s="55" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="M228" s="55"/>
       <c r="N228" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P228" s="86" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="S228" s="47"/>
       <c r="T228" s="47"/>
@@ -37105,7 +37134,7 @@
         <v>891</v>
       </c>
       <c r="L234" s="55" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="M234" s="55"/>
       <c r="N234" s="47" t="s">
@@ -37156,14 +37185,14 @@
         <v>1824</v>
       </c>
       <c r="L235" s="52" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="M235" s="52"/>
       <c r="N235" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P235" s="86" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="S235" s="47"/>
       <c r="T235" s="47"/>
@@ -37458,7 +37487,7 @@
         <v>1124</v>
       </c>
       <c r="L241" s="52" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="M241" s="52"/>
       <c r="N241" s="47" t="s">
@@ -37538,10 +37567,10 @@
         <v>900</v>
       </c>
       <c r="F243" s="66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G243" s="66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H243" s="65">
         <f t="shared" si="18"/>
@@ -37553,18 +37582,18 @@
       </c>
       <c r="J243" s="65">
         <f t="shared" si="19"/>
-        <v>545</v>
+        <v>1090</v>
       </c>
       <c r="K243" s="65">
         <f t="shared" si="20"/>
-        <v>545</v>
+        <v>0</v>
       </c>
       <c r="L243" s="52" t="s">
-        <v>1277</v>
+        <v>1366</v>
       </c>
       <c r="M243" s="52"/>
       <c r="N243" s="47" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="P243" s="86" t="s">
         <v>1254</v>
@@ -38042,7 +38071,7 @@
         <v>1239</v>
       </c>
       <c r="B249" s="52" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="C249" s="52" t="s">
         <v>95</v>
@@ -38081,17 +38110,17 @@
         <v>678</v>
       </c>
       <c r="P249" s="86" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="S249" s="47"/>
       <c r="T249" s="47"/>
     </row>
     <row r="250" spans="1:246" ht="17">
       <c r="A250" s="55" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B250" s="55" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="C250" s="55" t="s">
         <v>95</v>
@@ -38130,17 +38159,17 @@
         <v>678</v>
       </c>
       <c r="P250" s="86" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="S250" s="47"/>
       <c r="T250" s="47"/>
     </row>
     <row r="251" spans="1:246" ht="16">
       <c r="A251" s="52" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B251" s="52" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="C251" s="52" t="s">
         <v>96</v>
@@ -38177,7 +38206,7 @@
         <v>678</v>
       </c>
       <c r="O251" s="47" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="P251" s="86"/>
       <c r="S251" s="47"/>
@@ -38185,10 +38214,10 @@
     </row>
     <row r="252" spans="1:246" ht="16">
       <c r="A252" s="55" t="s">
+        <v>1338</v>
+      </c>
+      <c r="B252" s="55" t="s">
         <v>1339</v>
-      </c>
-      <c r="B252" s="55" t="s">
-        <v>1340</v>
       </c>
       <c r="C252" s="55" t="s">
         <v>96</v>
@@ -38225,7 +38254,7 @@
         <v>678</v>
       </c>
       <c r="O252" s="47" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="P252" s="86"/>
       <c r="S252" s="47"/>
@@ -38233,10 +38262,10 @@
     </row>
     <row r="253" spans="1:246" ht="16">
       <c r="A253" s="52" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B253" s="52" t="s">
         <v>1342</v>
-      </c>
-      <c r="B253" s="52" t="s">
-        <v>1343</v>
       </c>
       <c r="C253" s="52" t="s">
         <v>96</v>
@@ -38273,7 +38302,7 @@
         <v>678</v>
       </c>
       <c r="O253" s="47" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="P253" s="86"/>
       <c r="S253" s="47"/>
@@ -38281,10 +38310,10 @@
     </row>
     <row r="254" spans="1:246" ht="16">
       <c r="A254" s="55" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B254" s="55" t="s">
         <v>1344</v>
-      </c>
-      <c r="B254" s="55" t="s">
-        <v>1345</v>
       </c>
       <c r="C254" s="55" t="s">
         <v>96</v>
@@ -38321,7 +38350,7 @@
         <v>678</v>
       </c>
       <c r="O254" s="47" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="P254" s="86"/>
       <c r="S254" s="47"/>
@@ -38329,10 +38358,10 @@
     </row>
     <row r="255" spans="1:246" ht="16">
       <c r="A255" s="52" t="s">
+        <v>1348</v>
+      </c>
+      <c r="B255" s="52" t="s">
         <v>1349</v>
-      </c>
-      <c r="B255" s="52" t="s">
-        <v>1350</v>
       </c>
       <c r="C255" s="52" t="s">
         <v>95</v>
@@ -38366,7 +38395,7 @@
         <v>3564</v>
       </c>
       <c r="L255" s="52" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="M255" s="52"/>
       <c r="N255" s="47" t="s">
@@ -38378,10 +38407,10 @@
     </row>
     <row r="256" spans="1:246" ht="16">
       <c r="A256" s="55" t="s">
+        <v>1352</v>
+      </c>
+      <c r="B256" s="55" t="s">
         <v>1353</v>
-      </c>
-      <c r="B256" s="55" t="s">
-        <v>1354</v>
       </c>
       <c r="C256" s="55" t="s">
         <v>95</v>
@@ -38415,7 +38444,7 @@
         <v>1782</v>
       </c>
       <c r="L256" s="55" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="M256" s="55"/>
       <c r="N256" s="47" t="s">
@@ -44900,7 +44929,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>479698</v>
+        <v>483698</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -44908,11 +44937,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>182886.90339999998</v>
+        <v>184220.50339999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>296811.09660000005</v>
+        <v>299477.49660000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44920,7 +44949,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>159501.07060000004</v>
+        <v>162167.4706</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -44937,11 +44966,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>182777.19320000001</v>
+        <v>184109.9932</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-127454.19320000001</v>
+        <v>-128786.9932</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44949,7 +44978,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-55867.151200000008</v>
+        <v>-57199.951199999996</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -44966,11 +44995,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>182886.90339999998</v>
+        <v>184220.50339999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-170356.90339999998</v>
+        <v>-171690.50339999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44978,7 +45007,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-104633.91939999997</v>
+        <v>-105967.51939999998</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>